<commit_message>
Correcting start year date part 1
</commit_message>
<xml_diff>
--- a/InputData/elec/BBNPPTY/BAU Ban New Power Plants This Year.xlsx
+++ b/InputData/elec/BBNPPTY/BAU Ban New Power Plants This Year.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://energyinnovation.sharepoint.com/sites/IndonesiaEPS/Shared Documents/Updated Indonesia InputData files/elec/BBNPPTY/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mary Francis Swint\Vensim\eps-indonesia\InputData\elec\BBNPPTY\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{AC7CBECA-90CF-4BE3-9075-5F308FED293B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CE4AC36D-77D0-4824-8E89-E1F591B1E7EA}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4655730F-1F1E-4B98-82EC-88806A319DE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21825" yWindow="-5370" windowWidth="21795" windowHeight="19455" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="960" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -554,109 +554,112 @@
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
-  <dimension ref="A1:AE25"/>
+  <dimension ref="A1:AF25"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="26.453125" customWidth="1"/>
-    <col min="2" max="2" width="27.26953125" customWidth="1"/>
+    <col min="2" max="3" width="10.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B1">
+        <v>2020</v>
+      </c>
+      <c r="C1">
         <v>2021</v>
       </c>
-      <c r="C1">
+      <c r="D1">
         <v>2022</v>
       </c>
-      <c r="D1">
+      <c r="E1">
         <v>2023</v>
       </c>
-      <c r="E1">
+      <c r="F1">
         <v>2024</v>
       </c>
-      <c r="F1">
+      <c r="G1">
         <v>2025</v>
       </c>
-      <c r="G1">
+      <c r="H1">
         <v>2026</v>
       </c>
-      <c r="H1">
+      <c r="I1">
         <v>2027</v>
       </c>
-      <c r="I1">
+      <c r="J1">
         <v>2028</v>
       </c>
-      <c r="J1">
+      <c r="K1">
         <v>2029</v>
       </c>
-      <c r="K1">
+      <c r="L1">
         <v>2030</v>
       </c>
-      <c r="L1">
+      <c r="M1">
         <v>2031</v>
       </c>
-      <c r="M1">
+      <c r="N1">
         <v>2032</v>
       </c>
-      <c r="N1">
+      <c r="O1">
         <v>2033</v>
       </c>
-      <c r="O1">
+      <c r="P1">
         <v>2034</v>
       </c>
-      <c r="P1">
+      <c r="Q1">
         <v>2035</v>
       </c>
-      <c r="Q1">
+      <c r="R1">
         <v>2036</v>
       </c>
-      <c r="R1">
+      <c r="S1">
         <v>2037</v>
       </c>
-      <c r="S1">
+      <c r="T1">
         <v>2038</v>
       </c>
-      <c r="T1">
+      <c r="U1">
         <v>2039</v>
       </c>
-      <c r="U1">
+      <c r="V1">
         <v>2040</v>
       </c>
-      <c r="V1">
+      <c r="W1">
         <v>2041</v>
       </c>
-      <c r="W1">
+      <c r="X1">
         <v>2042</v>
       </c>
-      <c r="X1">
+      <c r="Y1">
         <v>2043</v>
       </c>
-      <c r="Y1">
+      <c r="Z1">
         <v>2044</v>
       </c>
-      <c r="Z1">
+      <c r="AA1">
         <v>2045</v>
       </c>
-      <c r="AA1">
+      <c r="AB1">
         <v>2046</v>
       </c>
-      <c r="AB1">
+      <c r="AC1">
         <v>2047</v>
       </c>
-      <c r="AC1">
+      <c r="AD1">
         <v>2048</v>
       </c>
-      <c r="AD1">
+      <c r="AE1">
         <v>2049</v>
       </c>
-      <c r="AE1">
+      <c r="AF1">
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -750,8 +753,11 @@
       <c r="AE2" s="5">
         <v>0</v>
       </c>
+      <c r="AF2" s="5">
+        <v>0</v>
+      </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>18</v>
       </c>
@@ -845,8 +851,11 @@
       <c r="AE3" s="5">
         <v>0</v>
       </c>
+      <c r="AF3" s="5">
+        <v>0</v>
+      </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>19</v>
       </c>
@@ -940,8 +949,11 @@
       <c r="AE4" s="5">
         <v>0</v>
       </c>
+      <c r="AF4" s="5">
+        <v>0</v>
+      </c>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -1035,8 +1047,11 @@
       <c r="AE5" s="5">
         <v>0</v>
       </c>
+      <c r="AF5" s="5">
+        <v>0</v>
+      </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>1</v>
       </c>
@@ -1130,8 +1145,11 @@
       <c r="AE6" s="5">
         <v>0</v>
       </c>
+      <c r="AF6" s="5">
+        <v>0</v>
+      </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -1225,8 +1243,11 @@
       <c r="AE7" s="5">
         <v>0</v>
       </c>
+      <c r="AF7" s="5">
+        <v>0</v>
+      </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -1320,8 +1341,11 @@
       <c r="AE8" s="5">
         <v>0</v>
       </c>
+      <c r="AF8" s="5">
+        <v>0</v>
+      </c>
     </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -1415,8 +1439,11 @@
       <c r="AE9" s="5">
         <v>0</v>
       </c>
+      <c r="AF9" s="5">
+        <v>0</v>
+      </c>
     </row>
-    <row r="10" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>2</v>
       </c>
@@ -1510,8 +1537,11 @@
       <c r="AE10" s="5">
         <v>0</v>
       </c>
+      <c r="AF10" s="5">
+        <v>0</v>
+      </c>
     </row>
-    <row r="11" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>7</v>
       </c>
@@ -1605,8 +1635,11 @@
       <c r="AE11" s="5">
         <v>0</v>
       </c>
+      <c r="AF11" s="5">
+        <v>0</v>
+      </c>
     </row>
-    <row r="12" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -1700,8 +1733,11 @@
       <c r="AE12" s="5">
         <v>0</v>
       </c>
+      <c r="AF12" s="5">
+        <v>0</v>
+      </c>
     </row>
-    <row r="13" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -1795,8 +1831,11 @@
       <c r="AE13" s="5">
         <v>0</v>
       </c>
+      <c r="AF13" s="5">
+        <v>0</v>
+      </c>
     </row>
-    <row r="14" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>10</v>
       </c>
@@ -1890,8 +1929,11 @@
       <c r="AE14" s="5">
         <v>0</v>
       </c>
+      <c r="AF14" s="5">
+        <v>0</v>
+      </c>
     </row>
-    <row r="15" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -1985,8 +2027,11 @@
       <c r="AE15" s="5">
         <v>0</v>
       </c>
+      <c r="AF15" s="5">
+        <v>0</v>
+      </c>
     </row>
-    <row r="16" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>14</v>
       </c>
@@ -2080,8 +2125,11 @@
       <c r="AE16" s="5">
         <v>0</v>
       </c>
+      <c r="AF16" s="5">
+        <v>0</v>
+      </c>
     </row>
-    <row r="17" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>15</v>
       </c>
@@ -2175,8 +2223,11 @@
       <c r="AE17" s="5">
         <v>0</v>
       </c>
+      <c r="AF17" s="5">
+        <v>0</v>
+      </c>
     </row>
-    <row r="18" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>16</v>
       </c>
@@ -2270,8 +2321,11 @@
       <c r="AE18" s="5">
         <v>0</v>
       </c>
+      <c r="AF18" s="5">
+        <v>0</v>
+      </c>
     </row>
-    <row r="19" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>20</v>
       </c>
@@ -2365,8 +2419,11 @@
       <c r="AE19" s="5">
         <v>0</v>
       </c>
+      <c r="AF19" s="5">
+        <v>0</v>
+      </c>
     </row>
-    <row r="20" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>21</v>
       </c>
@@ -2460,8 +2517,11 @@
       <c r="AE20" s="5">
         <v>0</v>
       </c>
+      <c r="AF20" s="5">
+        <v>0</v>
+      </c>
     </row>
-    <row r="21" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>22</v>
       </c>
@@ -2555,8 +2615,11 @@
       <c r="AE21" s="5">
         <v>0</v>
       </c>
+      <c r="AF21" s="5">
+        <v>0</v>
+      </c>
     </row>
-    <row r="22" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>23</v>
       </c>
@@ -2650,8 +2713,11 @@
       <c r="AE22" s="5">
         <v>0</v>
       </c>
+      <c r="AF22" s="5">
+        <v>0</v>
+      </c>
     </row>
-    <row r="23" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>24</v>
       </c>
@@ -2745,8 +2811,11 @@
       <c r="AE23" s="5">
         <v>0</v>
       </c>
+      <c r="AF23" s="5">
+        <v>0</v>
+      </c>
     </row>
-    <row r="24" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A24" s="6" t="s">
         <v>25</v>
       </c>
@@ -2840,8 +2909,11 @@
       <c r="AE24" s="5">
         <v>0</v>
       </c>
+      <c r="AF24" s="5">
+        <v>0</v>
+      </c>
     </row>
-    <row r="25" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A25" s="6" t="s">
         <v>26</v>
       </c>
@@ -2933,6 +3005,9 @@
         <v>0</v>
       </c>
       <c r="AE25" s="5">
+        <v>0</v>
+      </c>
+      <c r="AF25" s="5">
         <v>0</v>
       </c>
     </row>
@@ -2943,18 +3018,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3102,6 +3177,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{51DAAE7C-20DD-4D8B-9569-2359D66F2FCF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9E4BFBF7-F3C5-404B-A099-F047B4C5F933}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -3110,16 +3193,22 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{51DAAE7C-20DD-4D8B-9569-2359D66F2FCF}">
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F0AB0791-695F-4B71-8EA2-FE18F400AA1A}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="1659011e-6b88-4225-9a61-aaf33aaf19e8"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F0AB0791-695F-4B71-8EA2-FE18F400AA1A}"/>
 </file>
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>